<commit_message>
feat(academic): implement class and section academic structure feat(ai): add multilingual OCR extraction and AI language support feat(ui): redesign AI question generator interface
</commit_message>
<xml_diff>
--- a/smart_exam_system/static/downloads/student_import_template.xlsx
+++ b/smart_exam_system/static/downloads/student_import_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LMS_PROJECT\AI-Assessment-Platform\smart_exam_system\static\downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FCEE448-AE73-4406-A039-7FAB81BB30D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE51CA80-FE55-44F0-B1A4-D377BD63D93E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Instructions" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Students!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Students!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>First Name</t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>Sharma</t>
-  </si>
-  <si>
-    <t>8A</t>
   </si>
   <si>
     <t>Student Import Instructions</t>
@@ -117,12 +114,18 @@
   <si>
     <t>6. Save the file as .xlsx before importing.</t>
   </si>
+  <si>
+    <t>Section</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -157,6 +160,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -200,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -216,6 +227,12 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,16 +537,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="2" width="20.6328125" style="2" customWidth="1"/>
     <col min="3" max="3" width="12.6328125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="15.6328125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="18.6328125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="12.6328125" style="7" customWidth="1"/>
+    <col min="5" max="5" width="19.7265625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="18.6328125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" ht="15.5">
+    <row r="1" spans="1:6" s="3" customFormat="1" ht="15.5">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -539,32 +557,38 @@
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="C2" s="1">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="1">
         <v>15</v>
       </c>
-      <c r="E2" s="1">
+      <c r="F2" s="1">
         <v>9876543210</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -576,63 +600,63 @@
   <sheetData>
     <row r="1" spans="1:1" s="6" customFormat="1">
       <c r="A1" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:1" s="6" customFormat="1"/>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:1">
@@ -640,22 +664,22 @@
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>